<commit_message>
C12: two-layer conceptual graph (Ideas.layer, layer checks, trace targets, water-cycle mechanisms)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017xAqLftsSOeaVTWmpzXwHw
</commit_message>
<xml_diff>
--- a/fixtures/water-cycle/water-cycle.xlsx
+++ b/fixtures/water-cycle/water-cycle.xlsx
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -671,20 +671,25 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>layer</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>media_url</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>rarity</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>explanation</t>
         </is>
@@ -726,16 +731,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>water-cycle-overview.mp4</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>The journey water takes as it moves between the sky, the land and the sea, over and over again.</t>
         </is>
@@ -770,19 +779,27 @@
           <t>MS-ESS2-4, MS-PS1-4</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>thermal, phase</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>evaporation.mp4</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>When the Sun warms water in oceans, lakes and puddles, some of it turns into an invisible gas and rises into the air.</t>
         </is>
@@ -819,17 +836,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>evap</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+          <t>evap, phase</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>As water vapour rises it cools down and turns back into tiny drops of liquid water.</t>
         </is>
@@ -866,21 +886,25 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>cond</t>
+          <t>cond, dropmass, gravity</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>precipitation.mp4</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>When cloud drops grow too heavy, they fall back to the ground.</t>
         </is>
@@ -917,17 +941,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>prec</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
+          <t>prec, gravity, topo</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Water that falls gathers in oceans, rivers, lakes and underground, ready to start the cycle again.</t>
         </is>
@@ -967,14 +994,17 @@
           <t>plants</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Plants pull water up from their roots and let some of it escape from their leaves as vapour.</t>
         </is>
@@ -1014,14 +1044,17 @@
           <t>temp</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>When water gets cold enough it turns into solid ice.</t>
         </is>
@@ -1056,19 +1089,22 @@
           <t>MS-ESS2-4</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>sun-energy.mp4</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>The Sun gives off heat and light. Its energy is what keeps the water cycle moving.</t>
         </is>
@@ -1108,14 +1144,17 @@
           <t>sun</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>How hot or cold something is. Warm air can hold more water vapour than cold air.</t>
         </is>
@@ -1155,14 +1194,17 @@
           <t>temp, prec</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>The usual weather of a place over many years. It changes how much rain and snow falls.</t>
         </is>
@@ -1204,16 +1246,20 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>water-vapour.png</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Water in the form of a gas. You cannot see it, but it is all around you in the air.</t>
         </is>
@@ -1255,16 +1301,20 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>clouds.mp4</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Millions of tiny water drops or ice crystals floating together in the sky.</t>
         </is>
@@ -1294,20 +1344,22 @@
           <t>I can tell the difference between rain and snow.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>prec</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>The forms precipitation takes. Snow forms when the air is cold enough to freeze the drops.</t>
         </is>
@@ -1342,19 +1394,22 @@
           <t>MS-ESS2-6</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>oceans.jpg</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Huge bodies of salt water that cover most of the Earth and hold most of its water.</t>
         </is>
@@ -1394,14 +1449,17 @@
           <t>rain</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Flowing fresh water that carries rain and melted snow from the land back to the sea.</t>
         </is>
@@ -1436,15 +1494,17 @@
           <t>MS-LS1-6</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Living things that drink water through their roots and return some of it to the air.</t>
         </is>
@@ -1484,14 +1544,17 @@
           <t>ice</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Giant, slow rivers of ice that store fresh water for hundreds of years.</t>
         </is>
@@ -1531,16 +1594,284 @@
           <t>coll, aquifer</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Water that soaks into the soil and is stored between rocks underground.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Thermal energy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>I can explain that adding heat makes the tiny particles in water move faster.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>MS-PS1-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>thermal-energy.mp4</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Heat is the energy of tiny moving particles. The more thermal energy water has, the faster its particles move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Phase change</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>I can explain how adding or removing thermal energy changes water between solid, liquid and gas.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>MS-PS1-4</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>phase-change.mp4</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Water changes between ice, liquid and vapour when particles gain or lose enough thermal energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gravity</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>I can explain why gravity pulls water down toward the ground.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>MS-ESS2-4</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>gravity.mp4</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Gravity is the pull between the Earth and everything on it. It makes water fall and flow downhill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>dropmass</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Droplet mass</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>I can explain why a cloud drop falls only once it is heavy enough.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>MS-PS2-4</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>phase, gravity</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>droplet-mass.png</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Tiny drops stay up in the air. When many join together they get heavy enough for gravity to pull them down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>topo</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Topography</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>I can explain how the shape of the land decides where water flows and gathers.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MS-ESS2-2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>mechanism</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>topography.jpg</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Hills, valleys and slopes steer water downhill until it gathers in low places such as rivers, lakes and the sea.</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1679,7 +2010,6 @@
       <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1725,7 +2055,6 @@
       <c r="D7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1746,7 +2075,6 @@
       <c r="D8" t="n">
         <v>5</v>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1767,7 +2095,6 @@
       <c r="D9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1788,7 +2115,6 @@
       <c r="D10" t="n">
         <v>4</v>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1809,7 +2135,6 @@
       <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1830,7 +2155,6 @@
       <c r="D12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1851,7 +2175,6 @@
       <c r="D13" t="n">
         <v>4</v>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1872,7 +2195,6 @@
       <c r="D14" t="n">
         <v>4</v>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1893,7 +2215,6 @@
       <c r="D15" t="n">
         <v>3</v>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1914,7 +2235,6 @@
       <c r="D16" t="n">
         <v>2</v>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1935,7 +2255,6 @@
       <c r="D17" t="n">
         <v>4</v>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1956,7 +2275,6 @@
       <c r="D18" t="n">
         <v>4</v>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1977,7 +2295,6 @@
       <c r="D19" t="n">
         <v>4</v>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1998,7 +2315,6 @@
       <c r="D20" t="n">
         <v>3</v>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2019,7 +2335,6 @@
       <c r="D21" t="n">
         <v>4</v>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2040,7 +2355,6 @@
       <c r="D22" t="n">
         <v>3</v>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2061,7 +2375,6 @@
       <c r="D23" t="n">
         <v>3</v>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2082,7 +2395,6 @@
       <c r="D24" t="n">
         <v>4</v>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2103,7 +2415,6 @@
       <c r="D25" t="n">
         <v>4</v>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2124,7 +2435,6 @@
       <c r="D26" t="n">
         <v>3</v>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2145,7 +2455,6 @@
       <c r="D27" t="n">
         <v>3</v>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2166,7 +2475,6 @@
       <c r="D28" t="n">
         <v>3</v>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2187,7 +2495,6 @@
       <c r="D29" t="n">
         <v>3</v>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2208,7 +2515,6 @@
       <c r="D30" t="n">
         <v>2</v>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2229,7 +2535,6 @@
       <c r="D31" t="n">
         <v>2</v>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2250,7 +2555,246 @@
       <c r="D32" t="n">
         <v>2</v>
       </c>
-      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>evap</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>cond</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>rises and cools into</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cond</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>prec</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>leads to</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>prec</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>coll</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ends up in</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>coll</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>evap</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>feeds</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>evap</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>drives</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>sets off a</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>cond</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>explains</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>dropmass</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>builds</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>dropmass</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>prec</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>decides when</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>prec</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>pulls down</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>topo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>shapes</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>topo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>coll</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>steers water into</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2345,7 +2889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2727,6 +3271,106 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>Evaporation and condensation and precipitation and collection and and it repeats</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>thermal</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>What happens to water particles when they gain thermal energy?</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>They move faster, heat is the energy of moving particles</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>What happens to water when it gains enough thermal energy?</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>It changes phase, liquid water becomes a gas (vapour)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>gravity</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Why does water fall and flow downhill?</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Gravity pulls it toward the Earth, water follows the pull</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>dropmass</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Why do tiny cloud drops stay up until they grow?</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tiny drops are light, they fall only when heavy enough for gravity to win</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>topo</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>How does the shape of the land change where water goes?</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Water flows downhill, it gathers in low places like rivers and lakes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
C10: add the Practice tab (spec, contracts, import, data checks, diff and export)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017xAqLbwmkmFLWmDaNLDtEb
</commit_message>
<xml_diff>
--- a/fixtures/water-cycle/water-cycle.xlsx
+++ b/fixtures/water-cycle/water-cycle.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessment" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personas" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -734,7 +735,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>The journey water takes as it moves between the sky, the land and the sea, over and over again.</t>
@@ -770,7 +770,6 @@
           <t>MS-ESS2-4, MS-PS1-4</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>evaporation.mp4</t>
@@ -781,7 +780,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>When the Sun warms water in oceans, lakes and puddles, some of it turns into an invisible gas and rises into the air.</t>
@@ -822,13 +820,11 @@
           <t>evap</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>As water vapour rises it cools down and turns back into tiny drops of liquid water.</t>
@@ -879,7 +875,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>When cloud drops grow too heavy, they fall back to the ground.</t>
@@ -920,13 +915,11 @@
           <t>prec</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Water that falls gathers in oceans, rivers, lakes and underground, ready to start the cycle again.</t>
@@ -967,13 +960,11 @@
           <t>plants</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Plants pull water up from their roots and let some of it escape from their leaves as vapour.</t>
@@ -1014,13 +1005,11 @@
           <t>temp</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>When water gets cold enough it turns into solid ice.</t>
@@ -1056,7 +1045,6 @@
           <t>MS-ESS2-4</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>sun-energy.mp4</t>
@@ -1067,7 +1055,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>The Sun gives off heat and light. Its energy is what keeps the water cycle moving.</t>
@@ -1108,13 +1095,11 @@
           <t>sun</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>How hot or cold something is. Warm air can hold more water vapour than cold air.</t>
@@ -1155,13 +1140,11 @@
           <t>temp, prec</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>The usual weather of a place over many years. It changes how much rain and snow falls.</t>
@@ -1212,7 +1195,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>Water in the form of a gas. You cannot see it, but it is all around you in the air.</t>
@@ -1263,7 +1245,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>Millions of tiny water drops or ice crystals floating together in the sky.</t>
@@ -1294,19 +1275,16 @@
           <t>I can tell the difference between rain and snow.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>prec</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>The forms precipitation takes. Snow forms when the air is cold enough to freeze the drops.</t>
@@ -1342,7 +1320,6 @@
           <t>MS-ESS2-6</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>oceans.jpg</t>
@@ -1353,7 +1330,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>Huge bodies of salt water that cover most of the Earth and hold most of its water.</t>
@@ -1394,13 +1370,11 @@
           <t>rain</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>Flowing fresh water that carries rain and melted snow from the land back to the sea.</t>
@@ -1436,14 +1410,11 @@
           <t>MS-LS1-6</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>Living things that drink water through their roots and return some of it to the air.</t>
@@ -1484,13 +1455,11 @@
           <t>ice</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>Giant, slow rivers of ice that store fresh water for hundreds of years.</t>
@@ -1531,13 +1500,11 @@
           <t>coll, aquifer</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>Water that soaks into the soil and is stored between rocks underground.</t>
@@ -1679,7 +1646,6 @@
       <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1725,7 +1691,6 @@
       <c r="D7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1746,7 +1711,6 @@
       <c r="D8" t="n">
         <v>5</v>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1767,7 +1731,6 @@
       <c r="D9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1788,7 +1751,6 @@
       <c r="D10" t="n">
         <v>4</v>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1809,7 +1771,6 @@
       <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1830,7 +1791,6 @@
       <c r="D12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1851,7 +1811,6 @@
       <c r="D13" t="n">
         <v>4</v>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1872,7 +1831,6 @@
       <c r="D14" t="n">
         <v>4</v>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1893,7 +1851,6 @@
       <c r="D15" t="n">
         <v>3</v>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1914,7 +1871,6 @@
       <c r="D16" t="n">
         <v>2</v>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1935,7 +1891,6 @@
       <c r="D17" t="n">
         <v>4</v>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1956,7 +1911,6 @@
       <c r="D18" t="n">
         <v>4</v>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1977,7 +1931,6 @@
       <c r="D19" t="n">
         <v>4</v>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1998,7 +1951,6 @@
       <c r="D20" t="n">
         <v>3</v>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2019,7 +1971,6 @@
       <c r="D21" t="n">
         <v>4</v>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2040,7 +1991,6 @@
       <c r="D22" t="n">
         <v>3</v>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2061,7 +2011,6 @@
       <c r="D23" t="n">
         <v>3</v>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2082,7 +2031,6 @@
       <c r="D24" t="n">
         <v>4</v>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2103,7 +2051,6 @@
       <c r="D25" t="n">
         <v>4</v>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2124,7 +2071,6 @@
       <c r="D26" t="n">
         <v>3</v>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2145,7 +2091,6 @@
       <c r="D27" t="n">
         <v>3</v>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2166,7 +2111,6 @@
       <c r="D28" t="n">
         <v>3</v>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2187,7 +2131,6 @@
       <c r="D29" t="n">
         <v>3</v>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2208,7 +2151,6 @@
       <c r="D30" t="n">
         <v>2</v>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2229,7 +2171,6 @@
       <c r="D31" t="n">
         <v>2</v>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2250,7 +2191,6 @@
       <c r="D32" t="n">
         <v>2</v>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2991,4 +2931,486 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>exercise_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>idea_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>standard_code</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>exercise_title</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>quiz_from</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>problem_type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>choices</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>answer_unit</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>explanation</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>visual</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>media_url</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>demo_video_url</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>demo_steps</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>source_bank_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>license_type</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>attribution_string</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wc-evap-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>evap</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Evaporation and heat</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MS-PS1-4</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>What speeds up evaporation?</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>exercise</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>mc</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Which puddle dries fastest?</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>A shallow puddle in the sun | A deep puddle in the shade | A puddle on a cold night</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>A shallow puddle in the sun</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>More heat and more surface area both speed up evaporation.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>evaporation-demo.mp4</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Heat gives water molecules energy | The fastest ones escape the surface | A wider surface lets more escape | So a shallow puddle in the sun dries first</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wc-evap-1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>evap</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Evaporation and heat</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>MS-PS1-4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>What speeds up evaporation?</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>exercise</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>The graph shows how much water evaporates each hour at different temperatures (°C, mL). How many millilitres evaporate each hour at 30 °C?</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>mL</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Read up from 30 °C on the graph to the point (30, 9): 9 mL each hour.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>graph: 10,2; 20,5; 30,9; 40,14</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>wc-cond-1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cond</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Condensation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MS-ESS2-4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>How much vapour can air hold?</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>exercise</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>The table shows the most water vapour, in grams, that 1 m³ of air can hold at each temperature. How many more grams can it hold at 30 °C than at 20 °C?</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>30 °C holds 30 g and 20 °C holds 17 g, so 30 − 17 = 13 g more.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>table: temperature: 10, 20, 30; vapour: 9, 17, 30</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>vapour-table-hint.mp4</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>wc-cond-1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cond</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Condensation</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MS-ESS2-4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>How much vapour can air hold?</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>exercise</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>mc</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Warm, wet air rises and cools. What happens to the water vapour in it?</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>It condenses into tiny droplets | It evaporates faster | It turns into ice at once</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>It condenses into tiny droplets</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Cooler air holds less vapour, so the extra vapour turns back into liquid droplets.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Public Domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>wc-quiz-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cycle</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Water cycle review</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MS-ESS2-4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Water cycle quiz</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>wc-evap-1, wc-cond-1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>mc</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Which process turns water vapour back into liquid droplets?</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Condensation | Evaporation | Precipitation</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Condensation</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Condensation is vapour cooling into liquid; evaporation is the reverse.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Fixture Authors, Water Cycle Test Items, CC BY 4.0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>